<commit_message>
Expand regression suite for not in Spec and Pass but no evidence
</commit_message>
<xml_diff>
--- a/releases/2026.04/execution/Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx
+++ b/releases/2026.04/execution/Dynamic Scheduling and Optimisation Test Assurance Scripts v0.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david.watkin/Documents/Traceability_Reconciler_GeneralPurposeV5/releases/2026.04/execution/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEA88B9D-A645-5D45-8DA9-D4B620979965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1494EA36-6045-2A44-A170-FA199750E54F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5120" yWindow="25020" windowWidth="30420" windowHeight="16400" tabRatio="566" activeTab="2" xr2:uid="{C8155761-8FC3-4314-9FB8-C47B4CC04086}"/>
   </bookViews>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="826" uniqueCount="434">
   <si>
     <t>Document Information</t>
   </si>
@@ -2982,6 +2982,15 @@
   </si>
   <si>
     <t>Misalignment</t>
+  </si>
+  <si>
+    <t>STRY3999999</t>
+  </si>
+  <si>
+    <t>TP-ORPHAN-01</t>
+  </si>
+  <si>
+    <t>Not In Spec - no evidence</t>
   </si>
 </sst>
 </file>
@@ -3790,7 +3799,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="366">
+  <cellXfs count="367">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4747,6 +4756,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -4766,6 +4778,90 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4842,13 +4938,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -4885,279 +4974,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5262,7 +5078,175 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5339,7 +5323,28 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5403,6 +5408,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14393,27 +14405,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A42:B43 B44:D52 A44:A58 D53:D56 C57:D58">
-    <cfRule type="expression" dxfId="51" priority="55" stopIfTrue="1">
+    <cfRule type="expression" dxfId="51" priority="56" stopIfTrue="1">
+      <formula>($G42="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="50" priority="55" stopIfTrue="1">
       <formula>($G42="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="50" priority="56" stopIfTrue="1">
-      <formula>($G42="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A60:D65 C66:D66 A66:A131 B67:D68 C69:D70">
-    <cfRule type="expression" dxfId="49" priority="39" stopIfTrue="1">
+    <cfRule type="expression" dxfId="49" priority="40" stopIfTrue="1">
+      <formula>($G60="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="48" priority="39" stopIfTrue="1">
       <formula>($G60="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="48" priority="40" stopIfTrue="1">
-      <formula>($G60="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A21:G37">
-    <cfRule type="expression" dxfId="47" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="47" priority="2" stopIfTrue="1">
+      <formula>($G21="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="46" priority="1" stopIfTrue="1">
       <formula>($G21="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="46" priority="2" stopIfTrue="1">
-      <formula>($G21="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A59:G59">
@@ -14425,41 +14437,41 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13">
-    <cfRule type="expression" dxfId="43" priority="85" stopIfTrue="1">
+    <cfRule type="expression" dxfId="43" priority="88" stopIfTrue="1">
+      <formula>($G13="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="42" priority="87" stopIfTrue="1">
       <formula>($G13="Fail")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="86" stopIfTrue="1">
+    <cfRule type="expression" dxfId="41" priority="86" stopIfTrue="1">
       <formula>($G13="Pass")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="41" priority="87" stopIfTrue="1">
+    <cfRule type="expression" dxfId="40" priority="85" stopIfTrue="1">
       <formula>($G13="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="40" priority="88" stopIfTrue="1">
-      <formula>($G13="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:B15">
-    <cfRule type="expression" dxfId="39" priority="79" stopIfTrue="1">
+    <cfRule type="expression" dxfId="39" priority="80" stopIfTrue="1">
+      <formula>($G13="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="38" priority="79" stopIfTrue="1">
       <formula>($G13="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="38" priority="80" stopIfTrue="1">
-      <formula>($G13="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B13:B20">
-    <cfRule type="expression" dxfId="37" priority="95" stopIfTrue="1">
+    <cfRule type="expression" dxfId="37" priority="96" stopIfTrue="1">
+      <formula>($G13="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="36" priority="95" stopIfTrue="1">
       <formula>($G13="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="36" priority="96" stopIfTrue="1">
-      <formula>($G13="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B53:B58">
-    <cfRule type="expression" dxfId="35" priority="45" stopIfTrue="1">
+    <cfRule type="expression" dxfId="35" priority="46" stopIfTrue="1">
+      <formula>($G53="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="34" priority="45" stopIfTrue="1">
       <formula>($G53="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="34" priority="46" stopIfTrue="1">
-      <formula>($G53="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B66">
@@ -14479,27 +14491,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B38:C39">
-    <cfRule type="expression" dxfId="29" priority="63" stopIfTrue="1">
+    <cfRule type="expression" dxfId="29" priority="64" stopIfTrue="1">
+      <formula>($G38="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="28" priority="63" stopIfTrue="1">
       <formula>($G38="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="28" priority="64" stopIfTrue="1">
-      <formula>($G38="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B41:C41">
-    <cfRule type="expression" dxfId="27" priority="31" stopIfTrue="1">
+    <cfRule type="expression" dxfId="27" priority="32" stopIfTrue="1">
+      <formula>($G41="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="26" priority="31" stopIfTrue="1">
       <formula>($G41="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="26" priority="32" stopIfTrue="1">
-      <formula>($G41="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B40:F40">
-    <cfRule type="expression" dxfId="25" priority="19" stopIfTrue="1">
+    <cfRule type="expression" dxfId="25" priority="20" stopIfTrue="1">
+      <formula>($G40="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="24" priority="19" stopIfTrue="1">
       <formula>($G40="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="24" priority="20" stopIfTrue="1">
-      <formula>($G40="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C42">
@@ -14535,19 +14547,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C56">
-    <cfRule type="expression" dxfId="13" priority="47" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="48" stopIfTrue="1">
+      <formula>($G56="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="47" stopIfTrue="1">
       <formula>($G56="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="48" stopIfTrue="1">
-      <formula>($G56="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D41:D43">
-    <cfRule type="expression" dxfId="11" priority="17" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="18" stopIfTrue="1">
+      <formula>($G41="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="17" stopIfTrue="1">
       <formula>($G41="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="18" stopIfTrue="1">
-      <formula>($G41="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D38:F38">
@@ -14559,19 +14571,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E42:G58">
-    <cfRule type="expression" dxfId="7" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="7" priority="6" stopIfTrue="1">
+      <formula>($G42="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="5" stopIfTrue="1">
       <formula>($G42="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="6" stopIfTrue="1">
-      <formula>($G42="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E60:G70">
-    <cfRule type="expression" dxfId="5" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="12" stopIfTrue="1">
+      <formula>($G60="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="11" stopIfTrue="1">
       <formula>($G60="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="12" stopIfTrue="1">
-      <formula>($G60="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G6 A2:A20 D13:D20">
@@ -16833,7 +16845,33 @@
         <v>243</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="13.25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="14" spans="1:13" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="366" t="s">
+        <v>432</v>
+      </c>
+      <c r="B14" s="57" t="s">
+        <v>431</v>
+      </c>
+      <c r="C14" s="366" t="s">
+        <v>433</v>
+      </c>
+      <c r="D14" s="342" t="s">
+        <v>272</v>
+      </c>
+      <c r="E14" s="341" t="s">
+        <v>273</v>
+      </c>
+      <c r="F14" s="341" t="s">
+        <v>274</v>
+      </c>
+      <c r="G14" s="300">
+        <v>1</v>
+      </c>
+      <c r="H14" s="301"/>
+      <c r="I14" s="302" t="s">
+        <v>243</v>
+      </c>
+    </row>
     <row r="15" spans="1:13" ht="13.25" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="17" ht="13.25" customHeight="1" x14ac:dyDescent="0.15"/>
     <row r="18" ht="13.25" customHeight="1" x14ac:dyDescent="0.15"/>
@@ -23455,43 +23493,43 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A10:B10 A22:B22">
-    <cfRule type="expression" dxfId="92" priority="302" stopIfTrue="1">
+    <cfRule type="expression" dxfId="92" priority="303" stopIfTrue="1">
+      <formula>(#REF!="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="91" priority="302" stopIfTrue="1">
       <formula>(#REF!="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="91" priority="303" stopIfTrue="1">
-      <formula>(#REF!="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A11:B21">
-    <cfRule type="expression" dxfId="90" priority="290" stopIfTrue="1">
+    <cfRule type="expression" dxfId="90" priority="291" stopIfTrue="1">
+      <formula>($I10="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="89" priority="290" stopIfTrue="1">
       <formula>($I10="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="89" priority="291" stopIfTrue="1">
-      <formula>($I10="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A23:B26">
-    <cfRule type="expression" dxfId="88" priority="306" stopIfTrue="1">
+    <cfRule type="expression" dxfId="88" priority="307" stopIfTrue="1">
+      <formula>($I21="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="87" priority="306" stopIfTrue="1">
       <formula>($I21="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="87" priority="307" stopIfTrue="1">
-      <formula>($I21="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C5 C8:C9 C13:C21 D17:H17">
-    <cfRule type="expression" dxfId="86" priority="45" stopIfTrue="1">
+    <cfRule type="expression" dxfId="86" priority="46" stopIfTrue="1">
+      <formula>($I2="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="85" priority="45" stopIfTrue="1">
       <formula>($I2="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="85" priority="46" stopIfTrue="1">
-      <formula>($I2="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C29">
-    <cfRule type="expression" dxfId="84" priority="282" stopIfTrue="1">
+    <cfRule type="expression" dxfId="84" priority="283" stopIfTrue="1">
+      <formula>($I31="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="83" priority="282" stopIfTrue="1">
       <formula>($I31="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="83" priority="283" stopIfTrue="1">
-      <formula>($I31="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C30">
@@ -23503,11 +23541,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C33 F33">
-    <cfRule type="expression" dxfId="80" priority="286" stopIfTrue="1">
+    <cfRule type="expression" dxfId="80" priority="287" stopIfTrue="1">
+      <formula>($I34="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="79" priority="286" stopIfTrue="1">
       <formula>($I34="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="79" priority="287" stopIfTrue="1">
-      <formula>($I34="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D13:F16">
@@ -23551,11 +23589,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F34:F38">
-    <cfRule type="expression" dxfId="68" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="68" priority="4" stopIfTrue="1">
+      <formula>($I34="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="67" priority="3" stopIfTrue="1">
       <formula>($I34="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="67" priority="4" stopIfTrue="1">
-      <formula>($I34="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G12:H16">
@@ -23580,11 +23618,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J27">
-    <cfRule type="expression" dxfId="61" priority="19" stopIfTrue="1">
+    <cfRule type="expression" dxfId="61" priority="20" stopIfTrue="1">
+      <formula>($I29="Pass")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="60" priority="19" stopIfTrue="1">
       <formula>($I29="Fail")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="60" priority="20" stopIfTrue="1">
-      <formula>($I29="Pass")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -26239,12 +26277,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3b19dd56-76cb-4eb4-b732-a7bb000555f0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ebdbc82e-63f9-47eb-a0fa-eea99640aad4" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -26443,20 +26483,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3b19dd56-76cb-4eb4-b732-a7bb000555f0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ebdbc82e-63f9-47eb-a0fa-eea99640aad4" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E8101D3-AA49-4B42-B1EF-353911782D22}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11E644B2-2559-4456-96E7-5EC72762DBD4}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3b19dd56-76cb-4eb4-b732-a7bb000555f0"/>
+    <ds:schemaRef ds:uri="ebdbc82e-63f9-47eb-a0fa-eea99640aad4"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -26481,12 +26522,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11E644B2-2559-4456-96E7-5EC72762DBD4}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E8101D3-AA49-4B42-B1EF-353911782D22}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3b19dd56-76cb-4eb4-b732-a7bb000555f0"/>
-    <ds:schemaRef ds:uri="ebdbc82e-63f9-47eb-a0fa-eea99640aad4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>